<commit_message>
chore(research): refresh curated international discovery catalogue
</commit_message>
<xml_diff>
--- a/research/international-provider-candidates.xlsx
+++ b/research/international-provider-candidates.xlsx
@@ -312,7 +312,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -892,7 +892,7 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -964,25 +964,25 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CCLM</t>
+          <t>CNTV Play</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>movie,archive</t>
+          <t>movie,tv,documentary</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G16">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.cclm.cl/</t>
+          <t>https://cntvplay.cl/portada/</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -992,55 +992,55 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>archive</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Chilean archive candidate; kept for country coverage.</t>
+          <t>Official free Chilean streaming platform with more than 150 series plus films; geographically restricted to Chile.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://fmhy.net/non-english</t>
+          <t>https://cntvplay.cl/portada/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>16</v>
+        <v>97</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chine / sinophone</t>
+          <t>Chili</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>zh</t>
+          <t>es</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MoMoVOD</t>
+          <t>CCLM</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie,archive</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G17">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://momovod.app/</t>
+          <t>https://www.cclm.cl/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>archive</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Chilean archive candidate; kept for country coverage.</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1066,7 +1066,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>VidHub</t>
+          <t>MoMoVOD</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1094,11 +1094,11 @@
         </is>
       </c>
       <c r="G18">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://vidhub.me/</t>
+          <t>https://momovod.app/</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1124,7 +1124,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>xiaobaotv</t>
+          <t>VidHub</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1148,15 +1148,15 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G19">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.xiaobaotv.com/</t>
+          <t>https://vidhub.me/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1182,26 +1182,26 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Colombie</t>
+          <t>Chine / sinophone</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>zh</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>RTVCPlay</t>
+          <t>xiaobaotv</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>tv,public</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1210,11 +1210,11 @@
         </is>
       </c>
       <c r="G20">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://rtvcplay.co/</t>
+          <t>https://www.xiaobaotv.com/</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1224,12 +1224,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Public Colombian catalogue; useful country-coverage candidate.</t>
+          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1240,7 +1240,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1254,25 +1254,25 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Retina Latina</t>
+          <t>RTVCPlay</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>movie,documentary</t>
+          <t>tv,public</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G21">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.retinalatina.org/</t>
+          <t>https://rtvcplay.co/</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1282,12 +1282,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>regional-official</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Regional Latin American catalogue; lower general breadth but useful coverage.</t>
+          <t>Public Colombian catalogue; useful country-coverage candidate.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1298,39 +1298,39 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Corée du Sud</t>
+          <t>Colombie</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ko</t>
+          <t>es</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>OnDemandKorea</t>
+          <t>Retina Latina</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,documentary</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G22">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.ondemandkorea.com/</t>
+          <t>https://www.retinalatina.org/</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1340,12 +1340,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>regional-official</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Strong Korean catalogue candidate; assess geo/session requirements.</t>
+          <t>Regional Latin American catalogue; lower general breadth but useful coverage.</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1356,39 +1356,39 @@
     </row>
     <row r="23">
       <c r="A23">
+        <v>59</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Corée du Sud</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ko</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>OnDemandKorea</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>movie,tv</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G23">
         <v>88</v>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Corée du Sud</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>ko</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>AQ Stream</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>tv,live</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G23">
-        <v>82</v>
-      </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://aqstream.com/</t>
+          <t>https://www.ondemandkorea.com/</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1398,12 +1398,12 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Live-oriented candidate; verify VOD usefulness.</t>
+          <t>Strong Korean catalogue candidate; assess geo/session requirements.</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1414,7 +1414,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1428,25 +1428,25 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Naver TV</t>
+          <t>AQ Stream</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>tv,video</t>
+          <t>tv,live</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G24">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://tv.naver.com/</t>
+          <t>https://aqstream.com/</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1456,12 +1456,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Broad video platform; lower priority than direct VOD catalogues.</t>
+          <t>Live-oriented candidate; verify VOD usefulness.</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -1472,54 +1472,54 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Espagne</t>
+          <t>Corée du Sud</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>ko</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>HDFull</t>
+          <t>Naver TV</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>tv,video</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G25">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://dominioshdfull.com/</t>
+          <t>https://tv.naver.com/</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://dominioshdfull.com/</t>
+          <t/>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>domain-hub</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Strong candidate: the domain endpoint is itself intended to track the current HDFull address.</t>
+          <t>Broad video platform; lower priority than direct VOD catalogues.</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -1530,7 +1530,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Series.ly</t>
+          <t>HDFull</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1558,26 +1558,26 @@
         </is>
       </c>
       <c r="G26">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://series.ly/</t>
+          <t>https://dominioshdfull.com/</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://enlaces.ly/</t>
+          <t>https://dominioshdfull.com/</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>domain-hub</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Strong candidate: dedicated stable link/status endpoint available.</t>
+          <t>Strong candidate: the domain endpoint is itself intended to track the current HDFull address.</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -1588,7 +1588,7 @@
     </row>
     <row r="27">
       <c r="A27">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Cinezo</t>
+          <t>Series.ly</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1616,26 +1616,26 @@
         </is>
       </c>
       <c r="G27">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.cinezo.org/</t>
+          <t>https://series.ly/</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t/>
+          <t>https://enlaces.ly/</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>status</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Strong candidate: dedicated stable link/status endpoint available.</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -1646,7 +1646,7 @@
     </row>
     <row r="28">
       <c r="A28">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1660,25 +1660,25 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Tubepelis</t>
+          <t>Cinezo</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G28">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.tubepelis.com/</t>
+          <t>https://www.cinezo.org/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1704,21 +1704,21 @@
     </row>
     <row r="29">
       <c r="A29">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Finlande</t>
+          <t>Espagne</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>fi</t>
+          <t>es</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Areena</t>
+          <t>Tubepelis</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1732,11 +1732,11 @@
         </is>
       </c>
       <c r="G29">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://areena.yle.fi/</t>
+          <t>https://www.tubepelis.com/</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1746,12 +1746,12 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Official/free catalogue candidate; evaluate API/scrape feasibility and geo constraints.</t>
+          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -1762,7 +1762,7 @@
     </row>
     <row r="30">
       <c r="A30">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1776,25 +1776,25 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Elonet</t>
+          <t>Areena</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>movie</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G30">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://elonet.finna.fi/</t>
+          <t>https://areena.yle.fi/</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1804,12 +1804,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>archive</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Archive candidate; useful for country coverage, lower general-catalogue breadth.</t>
+          <t>Official/free catalogue candidate; evaluate API/scrape feasibility and geo constraints.</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -1820,7 +1820,7 @@
     </row>
     <row r="31">
       <c r="A31">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1834,12 +1834,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>TVKaista</t>
+          <t>Elonet</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>tv</t>
+          <t>movie</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1848,11 +1848,11 @@
         </is>
       </c>
       <c r="G31">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.tvkaista.org/</t>
+          <t>https://elonet.finna.fi/</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1862,12 +1862,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>iptv</t>
+          <t>archive</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Secondary TV candidate; verify VOD compatibility before onboarding.</t>
+          <t>Archive candidate; useful for country coverage, lower general-catalogue breadth.</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -1878,39 +1878,39 @@
     </row>
     <row r="32">
       <c r="A32">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Finlande</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>fi</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>OpenFlix</t>
+          <t>TVKaista</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>tv</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G32">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://openflix.pro/</t>
+          <t>https://www.tvkaista.org/</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1920,12 +1920,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>iptv</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Secondary TV candidate; verify VOD compatibility before onboarding.</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -1936,7 +1936,7 @@
     </row>
     <row r="33">
       <c r="A33">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Aether</t>
+          <t>OpenFlix</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1960,15 +1960,15 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G33">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://aether.ist/</t>
+          <t>https://openflix.pro/</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1994,7 +1994,7 @@
     </row>
     <row r="34">
       <c r="A34">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2008,12 +2008,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Bowd</t>
+          <t>Aether</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>movie,tv,live</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://bowdtv.com/</t>
+          <t>https://aether.ist/</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2052,21 +2052,21 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Grèce</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>el</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Greek-Movies</t>
+          <t>Bowd</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2076,15 +2076,15 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G35">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://greek-movies.com/</t>
+          <t>https://bowdtv.com/</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2110,7 +2110,7 @@
     </row>
     <row r="36">
       <c r="A36">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2124,25 +2124,25 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>xrysoi</t>
+          <t>Greek-Movies</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,live</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G36">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://xrysoi.pro/</t>
+          <t>https://greek-movies.com/</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2168,7 +2168,7 @@
     </row>
     <row r="37">
       <c r="A37">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>filmatic</t>
+          <t>xrysoi</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2196,11 +2196,11 @@
         </is>
       </c>
       <c r="G37">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://filmatic.online/</t>
+          <t>https://xrysoi.pro/</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2226,21 +2226,21 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Hongrie</t>
+          <t>Grèce</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>hu</t>
+          <t>el</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>moviedrive</t>
+          <t>filmatic</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2250,15 +2250,15 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G38">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://moviedrive.hu/</t>
+          <t>https://filmatic.online/</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2284,7 +2284,7 @@
     </row>
     <row r="39">
       <c r="A39">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>hdmozi</t>
+          <t>moviedrive</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2312,11 +2312,11 @@
         </is>
       </c>
       <c r="G39">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://hdmozi.hu/</t>
+          <t>https://moviedrive.hu/</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2342,7 +2342,7 @@
     </row>
     <row r="40">
       <c r="A40">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2356,25 +2356,25 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>OnlineFilmekIngyen</t>
+          <t>hdmozi</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>movie</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G40">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.onlinefilmekingyen1.com/</t>
+          <t>https://hdmozi.hu/</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2400,39 +2400,39 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Inde</t>
+          <t>Hongrie</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>hi,en</t>
+          <t>hu</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CinemaOS</t>
+          <t>OnlineFilmekIngyen</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G41">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://cinemaos.live/</t>
+          <t>https://www.onlinefilmekingyen1.com/</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2458,7 +2458,7 @@
     </row>
     <row r="42">
       <c r="A42">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2472,12 +2472,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>MultiMovies</t>
+          <t>CinemaOS</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2486,11 +2486,11 @@
         </is>
       </c>
       <c r="G42">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://multimovies.wtf/</t>
+          <t>https://cinemaos.live/</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2516,7 +2516,7 @@
     </row>
     <row r="43">
       <c r="A43">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2530,12 +2530,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1Tube</t>
+          <t>MultiMovies</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2544,11 +2544,11 @@
         </is>
       </c>
       <c r="G43">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.1tube.org/</t>
+          <t>https://multimovies.wtf/</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2574,7 +2574,7 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2583,30 +2583,30 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ta,hi,en</t>
+          <t>hi,en</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>TamilGun</t>
+          <t>1Tube</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G44">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://tamilgun.group/</t>
+          <t>https://www.1tube.org/</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2632,21 +2632,21 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Indonésie</t>
+          <t>Inde</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>ta,hi,en</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>idlixku</t>
+          <t>TamilGun</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2656,15 +2656,15 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G45">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://idlix.net/</t>
+          <t>https://tamilgun.group/</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2690,7 +2690,7 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>klikxxi</t>
+          <t>idlixku</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2718,11 +2718,11 @@
         </is>
       </c>
       <c r="G46">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://klikxxi.shop/</t>
+          <t>https://idlix.net/</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2748,7 +2748,7 @@
     </row>
     <row r="47">
       <c r="A47">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2762,25 +2762,25 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>OtakuDesu</t>
+          <t>klikxxi</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G47">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://otakudesu.cloud/</t>
+          <t>https://klikxxi.shop/</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2806,26 +2806,26 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Iran / persan</t>
+          <t>Indonésie</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>fa</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>RadioVatani</t>
+          <t>OtakuDesu</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>movie,tv,live</t>
+          <t>anime</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.radiovatani.com/</t>
+          <t>https://otakudesu.cloud/</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2864,7 +2864,7 @@
     </row>
     <row r="49">
       <c r="A49">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2878,12 +2878,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Nostalgik</t>
+          <t>RadioVatani</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>movie,tv,cartoon</t>
+          <t>movie,tv,live</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2892,11 +2892,11 @@
         </is>
       </c>
       <c r="G49">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://nostalgiktv.org/</t>
+          <t>https://www.radiovatani.com/</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2922,7 +2922,7 @@
     </row>
     <row r="50">
       <c r="A50">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>imvbox</t>
+          <t>Nostalgik</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,cartoon</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2950,11 +2950,11 @@
         </is>
       </c>
       <c r="G50">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.imvbox.com/</t>
+          <t>https://nostalgiktv.org/</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2980,26 +2980,26 @@
     </row>
     <row r="51">
       <c r="A51">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Israël</t>
+          <t>Iran / persan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>he</t>
+          <t>fa</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Animeil-TV</t>
+          <t>imvbox</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3012,7 +3012,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.animeil-tv.com/</t>
+          <t>https://www.imvbox.com/</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3038,7 +3038,7 @@
     </row>
     <row r="52">
       <c r="A52">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>aniplus</t>
+          <t>Animeil-TV</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3066,11 +3066,11 @@
         </is>
       </c>
       <c r="G52">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://aniplus.co/</t>
+          <t>https://www.animeil-tv.com/</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3096,7 +3096,7 @@
     </row>
     <row r="53">
       <c r="A53">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -3110,25 +3110,25 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>JFC</t>
+          <t>aniplus</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>movie,archive</t>
+          <t>anime</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G53">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://jfc.org.il/</t>
+          <t>https://aniplus.co/</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>archive</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Archive candidate; useful for local catalogue coverage.</t>
+          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -3154,54 +3154,54 @@
     </row>
     <row r="54">
       <c r="A54">
-        <v>3</v>
+        <v>95</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Italie</t>
+          <t>Israël</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>he</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>StreamingCommunity</t>
+          <t>JFC</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,archive</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G54">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://streamingcommunityz.red/</t>
+          <t>https://jfc.org.il/</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://telegra.ph/Link-Aggiornato-StreamingCommunity-09-29</t>
+          <t/>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>status-page</t>
+          <t>archive</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Strong candidate: persistent Telegraph address page can act as resolver hub.</t>
+          <t>Archive candidate; useful for local catalogue coverage.</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -3212,7 +3212,7 @@
     </row>
     <row r="55">
       <c r="A55">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -3226,12 +3226,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>StreamingUnity</t>
+          <t>StreamingCommunity</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3240,37 +3240,37 @@
         </is>
       </c>
       <c r="G55">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://streamingunity.vip/</t>
+          <t>https://streamingcommunityz.tax/</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t/>
+          <t>https://telegra.ph/Link-Aggiornato-StreamingCommunity-09-29</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>status-page</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Stable Telegraph address page used as resolver hub; terminal route updated from the page and must still be runtime-validated.</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://fmhy.net/non-english</t>
+          <t>https://telegra.ph/Link-Aggiornato-StreamingCommunity-09-29</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -3284,12 +3284,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>CB01</t>
+          <t>StreamingUnity</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3298,11 +3298,11 @@
         </is>
       </c>
       <c r="G56">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://cb01uno.homes/</t>
+          <t>https://streamingunity.vip/</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3328,7 +3328,7 @@
     </row>
     <row r="57">
       <c r="A57">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -3342,12 +3342,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>AnimeSaturn</t>
+          <t>CB01</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3356,26 +3356,26 @@
         </is>
       </c>
       <c r="G57">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.animesaturn.cx/</t>
+          <t>https://cb01uno.homes/</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://www.animesaturn.me/</t>
+          <t/>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>mirror</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Mirror/reference URL available; verify which endpoint is stable enough for hub use.</t>
+          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -3386,54 +3386,54 @@
     </row>
     <row r="58">
       <c r="A58">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Japon</t>
+          <t>Italie</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>it</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Abema</t>
+          <t>AnimeSaturn</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>tv,live</t>
+          <t>anime</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G58">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://abema.tv/</t>
+          <t>https://www.animesaturn.cx/</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t/>
+          <t>https://www.animesaturn.me/</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>mirror</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Official/free catalogue candidate; evaluate API/scrape feasibility and geo constraints.</t>
+          <t>Mirror/reference URL available; verify which endpoint is stable enough for hub use.</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -3444,7 +3444,7 @@
     </row>
     <row r="59">
       <c r="A59">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>JapanTV</t>
+          <t>Abema</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3472,11 +3472,11 @@
         </is>
       </c>
       <c r="G59">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://japantv.app/</t>
+          <t>https://abema.tv/</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3486,12 +3486,12 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Country-coverage candidate; verify VOD catalogue compatibility.</t>
+          <t>Official/free catalogue candidate; evaluate API/scrape feasibility and geo constraints.</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -3502,7 +3502,7 @@
     </row>
     <row r="60">
       <c r="A60">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -3516,12 +3516,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>NicoVideo</t>
+          <t>JapanTV</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>tv,live</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3530,11 +3530,11 @@
         </is>
       </c>
       <c r="G60">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.nicovideo.jp/</t>
+          <t>https://japantv.app/</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3544,12 +3544,12 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Broad video platform rather than a normal movie provider; lower onboarding priority.</t>
+          <t>Country-coverage candidate; verify VOD catalogue compatibility.</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -3560,26 +3560,26 @@
     </row>
     <row r="61">
       <c r="A61">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ouzbékistan</t>
+          <t>Japon</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>uz</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>uzmax.net</t>
+          <t>NicoVideo</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>video</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3588,11 +3588,11 @@
         </is>
       </c>
       <c r="G61">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://uzmax.net/</t>
+          <t>https://www.nicovideo.jp/</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3602,12 +3602,12 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Broad video platform rather than a normal movie provider; lower onboarding priority.</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -3618,7 +3618,7 @@
     </row>
     <row r="62">
       <c r="A62">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>AsilMedia</t>
+          <t>uzmax.net</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3646,11 +3646,11 @@
         </is>
       </c>
       <c r="G62">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://asilmedia.org/</t>
+          <t>https://uzmax.net/</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3676,39 +3676,39 @@
     </row>
     <row r="63">
       <c r="A63">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Ouzbékistan</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>fil</t>
+          <t>uz</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Movies Ni Pipay</t>
+          <t>AsilMedia</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G63">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://moviesnipipay.me/</t>
+          <t>https://asilmedia.org/</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3734,7 +3734,7 @@
     </row>
     <row r="64">
       <c r="A64">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Pinoy Movies Hub</t>
+          <t>Movies Ni Pipay</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3758,15 +3758,15 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G64">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://pinoymovieshub.cv/</t>
+          <t>https://moviesnipipay.me/</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3792,7 +3792,7 @@
     </row>
     <row r="65">
       <c r="A65">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -3806,12 +3806,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Pinoymoviepedia</t>
+          <t>Pinoy Movies Hub</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3820,11 +3820,11 @@
         </is>
       </c>
       <c r="G65">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://pinoymoviepedia.ru/</t>
+          <t>https://pinoymovieshub.cv/</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3850,21 +3850,21 @@
     </row>
     <row r="66">
       <c r="A66">
-        <v>7</v>
+        <v>81</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Pologne</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>fil</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Ekino-TV</t>
+          <t>Pinoymoviepedia</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3874,30 +3874,30 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G66">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://ekino.ws/</t>
+          <t>https://pinoymoviepedia.ru/</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://ekino-tv.link/</t>
+          <t/>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>mirror-index</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Strong candidate: dedicated mirror/index endpoint available.</t>
+          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -3908,7 +3908,7 @@
     </row>
     <row r="67">
       <c r="A67">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Filman</t>
+          <t>Ekino-TV</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3936,26 +3936,26 @@
         </is>
       </c>
       <c r="G67">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://filman.cc/</t>
+          <t>https://ekino.ws/</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t/>
+          <t>https://ekino-tv.link/</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>mirror-index</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Strong candidate: dedicated mirror/index endpoint available.</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -3966,7 +3966,7 @@
     </row>
     <row r="68">
       <c r="A68">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -3980,12 +3980,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Zaluknij</t>
+          <t>Filman</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3994,11 +3994,11 @@
         </is>
       </c>
       <c r="G68">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://zaluknij.cc/</t>
+          <t>https://filman.cc/</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4024,7 +4024,7 @@
     </row>
     <row r="69">
       <c r="A69">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>filmyonline</t>
+          <t>Zaluknij</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -4048,15 +4048,15 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G69">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://filmyonline.cc/</t>
+          <t>https://zaluknij.cc/</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4082,26 +4082,26 @@
     </row>
     <row r="70">
       <c r="A70">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Pérou</t>
+          <t>Pologne</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>pl</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Series Peruanas</t>
+          <t>filmyonline</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>tv,drama</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -4110,11 +4110,11 @@
         </is>
       </c>
       <c r="G70">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://seriesperu.com/</t>
+          <t>https://filmyonline.cc/</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Country-specific candidate; local source pool is sparse.</t>
+          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -4140,39 +4140,39 @@
     </row>
     <row r="71">
       <c r="A71">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Roumanie</t>
+          <t>Pérou</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>es</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>fsonline</t>
+          <t>Series Peruanas</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>tv,drama</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G71">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www3.fsonline.app/</t>
+          <t>https://seriesperu.com/</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Country-specific candidate; local source pool is sparse.</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -4198,39 +4198,39 @@
     </row>
     <row r="72">
       <c r="A72">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Roumanie</t>
+          <t>Pérou</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ro</t>
+          <t>es</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>VeziSeriale</t>
+          <t>TVPerú Play</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>tv,cultural,documentary</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G72">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://veziseriale.org/</t>
+          <t>https://www.tvperu.gob.pe/play</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -4240,23 +4240,23 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Official TVPerú streaming/program catalogue; country-coverage candidate with lower movie breadth.</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://fmhy.net/non-english</t>
+          <t>https://www.tvperu.gob.pe/play</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -4270,25 +4270,25 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>filmflix.ro</t>
+          <t>fsonline</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>movie</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G73">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://filmflix.ro/</t>
+          <t>https://www3.fsonline.app/</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4314,21 +4314,21 @@
     </row>
     <row r="74">
       <c r="A74">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Russie / RU</t>
+          <t>Roumanie</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Kinohub</t>
+          <t>VeziSeriale</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -4342,11 +4342,11 @@
         </is>
       </c>
       <c r="G74">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://on.kinohub.vip/</t>
+          <t>https://veziseriale.org/</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -4372,39 +4372,39 @@
     </row>
     <row r="75">
       <c r="A75">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Russie / RU</t>
+          <t>Roumanie</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>ro</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>KinoGo</t>
+          <t>filmflix.ro</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G75">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://kinogo.ec/</t>
+          <t>https://filmflix.ro/</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -4430,7 +4430,7 @@
     </row>
     <row r="76">
       <c r="A76">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -4444,12 +4444,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>KinoBase</t>
+          <t>Kinohub</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4458,11 +4458,11 @@
         </is>
       </c>
       <c r="G76">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://kinobase.org/</t>
+          <t>https://on.kinohub.vip/</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4488,7 +4488,7 @@
     </row>
     <row r="77">
       <c r="A77">
-        <v>68</v>
+        <v>15</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -4502,7 +4502,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>filmix</t>
+          <t>KinoGo</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4512,15 +4512,15 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G77">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://filmix.my/</t>
+          <t>https://kinogo.ec/</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4546,21 +4546,21 @@
     </row>
     <row r="78">
       <c r="A78">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Slovaquie</t>
+          <t>Russie / RU</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>sk</t>
+          <t>ru</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>tuu.to</t>
+          <t>KinoBase</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4570,15 +4570,15 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G78">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://tuu.to/</t>
+          <t>https://kinobase.org/</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4604,7 +4604,7 @@
     </row>
     <row r="79">
       <c r="A79">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>jOj Archive</t>
+          <t>tuu.to</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4628,15 +4628,15 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G79">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.joj.sk/</t>
+          <t>https://tuu.to/</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4646,12 +4646,12 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Country-coverage candidate; assess usable catalogue routes.</t>
+          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -4662,7 +4662,7 @@
     </row>
     <row r="80">
       <c r="A80">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Markiza</t>
+          <t>jOj Archive</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4690,11 +4690,11 @@
         </is>
       </c>
       <c r="G80">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.markiza.sk/</t>
+          <t>https://www.joj.sk/</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4720,21 +4720,21 @@
     </row>
     <row r="81">
       <c r="A81">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Suède</t>
+          <t>Slovaquie</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>sv</t>
+          <t>sk</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SVT Play</t>
+          <t>Markiza</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4744,15 +4744,15 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G81">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.svtplay.se/</t>
+          <t>https://www.markiza.sk/</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Official Swedish catalogue; evaluate geo/API constraints.</t>
+          <t>Country-coverage candidate; assess usable catalogue routes.</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -4778,7 +4778,7 @@
     </row>
     <row r="82">
       <c r="A82">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -4792,25 +4792,25 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Stockholmskallan</t>
+          <t>SVT Play</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>movie,archive</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G82">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://stockholmskallan.stockholm.se/</t>
+          <t>https://www.svtplay.se/</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4820,12 +4820,12 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>archive</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Public-domain archive; lower general-catalogue breadth.</t>
+          <t>Official Swedish catalogue; evaluate geo/API constraints.</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -4836,39 +4836,39 @@
     </row>
     <row r="83">
       <c r="A83">
-        <v>30</v>
+        <v>99</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Tchéquie</t>
+          <t>Suède</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>cs</t>
+          <t>sv</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Bombuj</t>
+          <t>Stockholmskallan</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,archive</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G83">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://bombuj.si/</t>
+          <t>https://stockholmskallan.stockholm.se/</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4878,12 +4878,12 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>archive</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Public-domain archive; lower general-catalogue breadth.</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -4894,7 +4894,7 @@
     </row>
     <row r="84">
       <c r="A84">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -4908,12 +4908,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Sledujteto</t>
+          <t>Bombuj</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4922,11 +4922,11 @@
         </is>
       </c>
       <c r="G84">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.sledujteto.cz/</t>
+          <t>https://bombuj.si/</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4952,7 +4952,7 @@
     </row>
     <row r="85">
       <c r="A85">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -4966,7 +4966,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>filmbot</t>
+          <t>Sledujteto</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4976,15 +4976,15 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G85">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://filmbot.tv/</t>
+          <t>https://www.sledujteto.cz/</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5010,21 +5010,21 @@
     </row>
     <row r="86">
       <c r="A86">
-        <v>1</v>
+        <v>67</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Turquie</t>
+          <t>Tchéquie</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>tr</t>
+          <t>cs</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Dizi Film Botu</t>
+          <t>filmbot</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -5034,30 +5034,30 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G86">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://t.me/Difix9Bot</t>
+          <t>https://filmbot.tv/</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://t.me/Difix9Bot</t>
+          <t/>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>telegram</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>High-value Telegram source: stable Telegram identity can serve as resolver source even when terminal domains rotate.</t>
+          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -5068,7 +5068,7 @@
     </row>
     <row r="87">
       <c r="A87">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -5082,12 +5082,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Dizipal</t>
+          <t>Dizi Film Botu</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>movie,tv</t>
+          <t>movie,tv,anime</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -5096,26 +5096,26 @@
         </is>
       </c>
       <c r="G87">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://dizipal1453.com/</t>
+          <t>https://t.me/Difix9Bot</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t/>
+          <t>https://t.me/Difix9Bot</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>High-value Telegram source: stable Telegram identity can serve as resolver source even when terminal domains rotate.</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -5126,7 +5126,7 @@
     </row>
     <row r="88">
       <c r="A88">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Dizilla</t>
+          <t>Dizipal</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -5154,11 +5154,11 @@
         </is>
       </c>
       <c r="G88">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://dizilla.to/</t>
+          <t>https://dizipal1453.com/</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -5184,7 +5184,7 @@
     </row>
     <row r="89">
       <c r="A89">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Hdfilmcehennemi</t>
+          <t>Dizilla</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -5208,15 +5208,15 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G89">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.hdfilmcehennemi.nl/</t>
+          <t>https://dizilla.to/</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -5242,39 +5242,39 @@
     </row>
     <row r="90">
       <c r="A90">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Turquie</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>uk</t>
+          <t>tr</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Kinostrain</t>
+          <t>Hdfilmcehennemi</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>movie,tv,anime</t>
+          <t>movie,tv</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G90">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://kinostrain.com/</t>
+          <t>https://www.hdfilmcehennemi.nl/</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -5300,7 +5300,7 @@
     </row>
     <row r="91">
       <c r="A91">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>UAKino-Bay</t>
+          <t>Kinostrain</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -5328,11 +5328,11 @@
         </is>
       </c>
       <c r="G91">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://uakino-bay.net/</t>
+          <t>https://kinostrain.com/</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -5358,7 +5358,7 @@
     </row>
     <row r="92">
       <c r="A92">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -5372,7 +5372,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>UASerials</t>
+          <t>UAKino-Bay</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -5386,11 +5386,11 @@
         </is>
       </c>
       <c r="G92">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://uaserials.my/</t>
+          <t>https://uakino-bay.net/</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -5416,21 +5416,21 @@
     </row>
     <row r="93">
       <c r="A93">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>vi</t>
+          <t>uk</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Tram Phim</t>
+          <t>UASerials</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -5444,11 +5444,11 @@
         </is>
       </c>
       <c r="G93">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://tramphim4.org/</t>
+          <t>https://uaserials.my/</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -5474,7 +5474,7 @@
     </row>
     <row r="94">
       <c r="A94">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -5488,7 +5488,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Sofaflix</t>
+          <t>Tram Phim</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -5502,11 +5502,11 @@
         </is>
       </c>
       <c r="G94">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://sofaflix.shop/</t>
+          <t>https://tramphim4.org/</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -5532,7 +5532,7 @@
     </row>
     <row r="95">
       <c r="A95">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -5546,7 +5546,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>kkphim</t>
+          <t>Sofaflix</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -5560,11 +5560,11 @@
         </is>
       </c>
       <c r="G95">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://kkphim.com/</t>
+          <t>https://sofaflix.shop/</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -5590,7 +5590,7 @@
     </row>
     <row r="96">
       <c r="A96">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>NguonC</t>
+          <t>kkphim</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -5618,11 +5618,11 @@
         </is>
       </c>
       <c r="G96">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://phim.nguonc.com/</t>
+          <t>https://kkphim.com/</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5822,39 +5822,39 @@
     </row>
     <row r="100">
       <c r="A100">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Égypte / MENA</t>
+          <t>Équateur</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>ar</t>
+          <t>es</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>FajerShow</t>
+          <t>Cinecalidad</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>movie,tv,cartoon</t>
+          <t>movie,tv,animation</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G100">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>https://fajer.show/</t>
+          <t>https://www.cinecalidad.ec/</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Curated candidate; validate identity, catalogue route and playable media before onboarding.</t>
+          <t>Strong country-specific candidate; only one sufficiently strong Ecuador entry retained.</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -5880,7 +5880,7 @@
     </row>
     <row r="101">
       <c r="A101">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -5894,25 +5894,25 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Cinecalidad</t>
+          <t>Ecuador TV</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>movie,tv,animation</t>
+          <t>tv,series,on-demand</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G101">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>https://www.cinecalidad.ec/</t>
+          <t>https://www.ecuadortv.ec/</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5922,17 +5922,17 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>official</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Strong country-specific candidate; only one sufficiently strong Ecuador entry retained.</t>
+          <t>Official Ecuador TV platform relaunched in February 2026 with live viewing and on-demand programmes; country-coverage candidate.</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://fmhy.net/non-english</t>
+          <t>https://www.ecuadortv.ec/</t>
         </is>
       </c>
     </row>
@@ -6090,17 +6090,17 @@
         </is>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SOURCE RARE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
         <v>4</v>
       </c>
       <c r="C20">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D20">
         <v>2</v>
@@ -6468,7 +6468,7 @@
         </is>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25">
         <v>84</v>
@@ -6478,7 +6478,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SOURCE RARE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -6510,7 +6510,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C27">
         <v>94</v>
@@ -6636,7 +6636,7 @@
         </is>
       </c>
       <c r="B33">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C33">
         <v>94</v>
@@ -6657,7 +6657,7 @@
         </is>
       </c>
       <c r="B34">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C34">
         <v>94</v>
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="B35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35">
         <v>91</v>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SOURCE RARE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-09T20:03:33.638422+00:00</t>
+          <t>2026-09-09T20:08:06.869178+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>